<commit_message>
refactor(pruebas): arquitectura por integrante, reto avanzado y CI multipropósito
Reorganiza las entregas en carpetas por integrante, agrega la ronda avanzada de 5 pruebas, endurece el contrato y la mutación por símbolo, mueve el Excel de 470 casos a docs/.interno (ignorado), prueba SQLite/PostgreSQL/MySQL en CI y bloquea main con checks obligatorios.
</commit_message>
<xml_diff>
--- a/docs/pruebas/Plan_de_Pruebas_PlomApp_SENA_entrega_equipo.xlsx
+++ b/docs/pruebas/Plan_de_Pruebas_PlomApp_SENA_entrega_equipo.xlsx
@@ -819,7 +819,6 @@
       </c>
     </row>
     <row r="2" ht="21.75" customHeight="1" s="45"/>
-    <row r="3"/>
     <row r="4" ht="19.5" customHeight="1" s="45">
       <c r="A4" s="47" t="inlineStr">
         <is>
@@ -932,7 +931,6 @@
       <c r="I7" s="49" t="n"/>
       <c r="J7" s="48" t="n"/>
     </row>
-    <row r="8"/>
     <row r="9" ht="21.75" customHeight="1" s="45">
       <c r="A9" s="50" t="inlineStr">
         <is>
@@ -940,7 +938,6 @@
         </is>
       </c>
     </row>
-    <row r="10"/>
     <row r="11" ht="18" customHeight="1" s="45">
       <c r="A11" s="51" t="inlineStr">
         <is>
@@ -1012,7 +1009,6 @@
       <c r="I13" s="55" t="n"/>
       <c r="J13" s="56" t="n"/>
     </row>
-    <row r="14"/>
     <row r="15" ht="21.75" customHeight="1" s="45">
       <c r="A15" s="50" t="inlineStr">
         <is>
@@ -2414,6 +2410,7 @@
       </c>
     </row>
     <row r="2" ht="21.75" customHeight="1" s="45"/>
+    <row r="3"/>
     <row r="4" ht="24" customHeight="1" s="45">
       <c r="A4" s="15" t="inlineStr">
         <is>
@@ -2489,7 +2486,7 @@
     <row r="6" ht="34" customHeight="1" s="45">
       <c r="A6" s="66" t="inlineStr">
         <is>
-          <t>ENTREGA ACTUAL: 20 PRUEBAS UNITARIAS de Andrés Durán y Dairon Salazar (UNIT-001 a UNIT-020), 10 por integrante en api/tests/unit/equipo/. Ejecución real: 20 passed. Las 20 pruebas de Sebastián Samacá y Kevin Pinzón quedan pendientes: deben escribir las suyas en archivos propios y no repetirlas.</t>
+          <t>ENTREGA ACTUAL: 20 PRUEBAS UNITARIAS base de Andr?s Dur?n y Dairon Salazar (UNIT-001 a UNIT-020), 10 por integrante en api/tests/unit/equipo/. Ejecuci?n real: 20 passed. Sebasti?n Samac? y Kevin Pinz?n tienen pendientes la ronda base; los 4 integrantes tienen pendiente la ronda avanzada (5 pruebas cada uno).</t>
         </is>
       </c>
     </row>
@@ -2583,7 +2580,7 @@
       </c>
       <c r="E8" s="69" t="inlineStr">
         <is>
-          <t>1. Ejecutar: pytest api\tests\unit\equipo\test_integrante_1_validaciones.py::test_email_valido
+          <t>1. Ejecutar: pytest api\tests\unit\equipo\integrante_1_validaciones\test_integrante_1_validaciones.py::test_email_valido
 2. validate_email("carlos@plomaap.com")</t>
         </is>
       </c>
@@ -2614,7 +2611,7 @@
       </c>
       <c r="K8" s="70" t="inlineStr">
         <is>
-          <t>api\tests\unit\equipo\test_integrante_1_validaciones.py::test_email_valido -&gt; 1 passed</t>
+          <t>api\tests\unit\equipo\integrante_1_validaciones\test_integrante_1_validaciones.py::test_email_valido -&gt; 1 passed</t>
         </is>
       </c>
       <c r="L8" s="69" t="inlineStr">
@@ -2651,7 +2648,7 @@
       </c>
       <c r="E9" s="73" t="inlineStr">
         <is>
-          <t>1. Ejecutar: pytest api\tests\unit\equipo\test_integrante_1_validaciones.py::test_email_sin_arroba_es_invalido
+          <t>1. Ejecutar: pytest api\tests\unit\equipo\integrante_1_validaciones\test_integrante_1_validaciones.py::test_email_sin_arroba_es_invalido
 2. validate_email("carlos.plomaap.com")</t>
         </is>
       </c>
@@ -2682,7 +2679,7 @@
       </c>
       <c r="K9" s="74" t="inlineStr">
         <is>
-          <t>api\tests\unit\equipo\test_integrante_1_validaciones.py::test_email_sin_arroba_es_invalido -&gt; 1 passed</t>
+          <t>api\tests\unit\equipo\integrante_1_validaciones\test_integrante_1_validaciones.py::test_email_sin_arroba_es_invalido -&gt; 1 passed</t>
         </is>
       </c>
       <c r="L9" s="73" t="inlineStr">
@@ -2719,7 +2716,7 @@
       </c>
       <c r="E10" s="73" t="inlineStr">
         <is>
-          <t>1. Ejecutar: pytest api\tests\unit\equipo\test_integrante_1_validaciones.py::test_password_de_ocho_caracteres_es_valida
+          <t>1. Ejecutar: pytest api\tests\unit\equipo\integrante_1_validaciones\test_integrante_1_validaciones.py::test_password_de_ocho_caracteres_es_valida
 2. validate_password("PlomApp1")</t>
         </is>
       </c>
@@ -2750,7 +2747,7 @@
       </c>
       <c r="K10" s="74" t="inlineStr">
         <is>
-          <t>api\tests\unit\equipo\test_integrante_1_validaciones.py::test_password_de_ocho_caracteres_es_valida -&gt; 1 passed</t>
+          <t>api\tests\unit\equipo\integrante_1_validaciones\test_integrante_1_validaciones.py::test_password_de_ocho_caracteres_es_valida -&gt; 1 passed</t>
         </is>
       </c>
       <c r="L10" s="73" t="inlineStr">
@@ -2787,7 +2784,7 @@
       </c>
       <c r="E11" s="73" t="inlineStr">
         <is>
-          <t>1. Ejecutar: pytest api\tests\unit\equipo\test_integrante_1_validaciones.py::test_password_corta_es_invalida
+          <t>1. Ejecutar: pytest api\tests\unit\equipo\integrante_1_validaciones\test_integrante_1_validaciones.py::test_password_corta_es_invalida
 2. validate_password("1234")</t>
         </is>
       </c>
@@ -2818,7 +2815,7 @@
       </c>
       <c r="K11" s="74" t="inlineStr">
         <is>
-          <t>api\tests\unit\equipo\test_integrante_1_validaciones.py::test_password_corta_es_invalida -&gt; 1 passed</t>
+          <t>api\tests\unit\equipo\integrante_1_validaciones\test_integrante_1_validaciones.py::test_password_corta_es_invalida -&gt; 1 passed</t>
         </is>
       </c>
       <c r="L11" s="73" t="inlineStr">
@@ -2855,7 +2852,7 @@
       </c>
       <c r="E12" s="73" t="inlineStr">
         <is>
-          <t>1. Ejecutar: pytest api\tests\unit\equipo\test_integrante_1_validaciones.py::test_telefono_valido
+          <t>1. Ejecutar: pytest api\tests\unit\equipo\integrante_1_validaciones\test_integrante_1_validaciones.py::test_telefono_valido
 2. validate_phone("+573001234567")</t>
         </is>
       </c>
@@ -2886,7 +2883,7 @@
       </c>
       <c r="K12" s="74" t="inlineStr">
         <is>
-          <t>api\tests\unit\equipo\test_integrante_1_validaciones.py::test_telefono_valido -&gt; 1 passed</t>
+          <t>api\tests\unit\equipo\integrante_1_validaciones\test_integrante_1_validaciones.py::test_telefono_valido -&gt; 1 passed</t>
         </is>
       </c>
       <c r="L12" s="73" t="inlineStr">
@@ -2923,7 +2920,7 @@
       </c>
       <c r="E13" s="73" t="inlineStr">
         <is>
-          <t>1. Ejecutar: pytest api\tests\unit\equipo\test_integrante_1_validaciones.py::test_telefono_con_letras_es_invalido
+          <t>1. Ejecutar: pytest api\tests\unit\equipo\integrante_1_validaciones\test_integrante_1_validaciones.py::test_telefono_con_letras_es_invalido
 2. validate_phone("abc1234567")</t>
         </is>
       </c>
@@ -2954,7 +2951,7 @@
       </c>
       <c r="K13" s="74" t="inlineStr">
         <is>
-          <t>api\tests\unit\equipo\test_integrante_1_validaciones.py::test_telefono_con_letras_es_invalido -&gt; 1 passed</t>
+          <t>api\tests\unit\equipo\integrante_1_validaciones\test_integrante_1_validaciones.py::test_telefono_con_letras_es_invalido -&gt; 1 passed</t>
         </is>
       </c>
       <c r="L13" s="73" t="inlineStr">
@@ -2991,7 +2988,7 @@
       </c>
       <c r="E14" s="73" t="inlineStr">
         <is>
-          <t>1. Ejecutar: pytest api\tests\unit\equipo\test_integrante_1_validaciones.py::test_nombre_de_un_caracter_es_invalido
+          <t>1. Ejecutar: pytest api\tests\unit\equipo\integrante_1_validaciones\test_integrante_1_validaciones.py::test_nombre_de_un_caracter_es_invalido
 2. validate_name("A")</t>
         </is>
       </c>
@@ -3022,7 +3019,7 @@
       </c>
       <c r="K14" s="74" t="inlineStr">
         <is>
-          <t>api\tests\unit\equipo\test_integrante_1_validaciones.py::test_nombre_de_un_caracter_es_invalido -&gt; 1 passed</t>
+          <t>api\tests\unit\equipo\integrante_1_validaciones\test_integrante_1_validaciones.py::test_nombre_de_un_caracter_es_invalido -&gt; 1 passed</t>
         </is>
       </c>
       <c r="L14" s="73" t="inlineStr">
@@ -3059,7 +3056,7 @@
       </c>
       <c r="E15" s="73" t="inlineStr">
         <is>
-          <t>1. Ejecutar: pytest api\tests\unit\equipo\test_integrante_1_validaciones.py::test_fecha_y_hora_validas
+          <t>1. Ejecutar: pytest api\tests\unit\equipo\integrante_1_validaciones\test_integrante_1_validaciones.py::test_fecha_y_hora_validas
 2. validate_date_time("2026-11-02", "09:30")</t>
         </is>
       </c>
@@ -3090,7 +3087,7 @@
       </c>
       <c r="K15" s="74" t="inlineStr">
         <is>
-          <t>api\tests\unit\equipo\test_integrante_1_validaciones.py::test_fecha_y_hora_validas -&gt; 1 passed</t>
+          <t>api\tests\unit\equipo\integrante_1_validaciones\test_integrante_1_validaciones.py::test_fecha_y_hora_validas -&gt; 1 passed</t>
         </is>
       </c>
       <c r="L15" s="73" t="inlineStr">
@@ -3127,7 +3124,7 @@
       </c>
       <c r="E16" s="73" t="inlineStr">
         <is>
-          <t>1. Ejecutar: pytest api\tests\unit\equipo\test_integrante_1_validaciones.py::test_fecha_con_formato_incorrecto_es_invalida
+          <t>1. Ejecutar: pytest api\tests\unit\equipo\integrante_1_validaciones\test_integrante_1_validaciones.py::test_fecha_con_formato_incorrecto_es_invalida
 2. validate_date_time("02/11/2026", "09:30")</t>
         </is>
       </c>
@@ -3158,7 +3155,7 @@
       </c>
       <c r="K16" s="74" t="inlineStr">
         <is>
-          <t>api\tests\unit\equipo\test_integrante_1_validaciones.py::test_fecha_con_formato_incorrecto_es_invalida -&gt; 1 passed</t>
+          <t>api\tests\unit\equipo\integrante_1_validaciones\test_integrante_1_validaciones.py::test_fecha_con_formato_incorrecto_es_invalida -&gt; 1 passed</t>
         </is>
       </c>
       <c r="L16" s="73" t="inlineStr">
@@ -3195,7 +3192,7 @@
       </c>
       <c r="E17" s="73" t="inlineStr">
         <is>
-          <t>1. Ejecutar: pytest api\tests\unit\equipo\test_integrante_1_validaciones.py::test_rol_valido
+          <t>1. Ejecutar: pytest api\tests\unit\equipo\integrante_1_validaciones\test_integrante_1_validaciones.py::test_rol_valido
 2. validate_role("technician")</t>
         </is>
       </c>
@@ -3226,7 +3223,7 @@
       </c>
       <c r="K17" s="74" t="inlineStr">
         <is>
-          <t>api\tests\unit\equipo\test_integrante_1_validaciones.py::test_rol_valido -&gt; 1 passed</t>
+          <t>api\tests\unit\equipo\integrante_1_validaciones\test_integrante_1_validaciones.py::test_rol_valido -&gt; 1 passed</t>
         </is>
       </c>
       <c r="L17" s="73" t="inlineStr">
@@ -3263,7 +3260,7 @@
       </c>
       <c r="E18" s="73" t="inlineStr">
         <is>
-          <t>1. Ejecutar: pytest api\tests\unit\equipo\test_integrante_3_citas.py::test_pendiente_puede_pasar_a_agendada
+          <t>1. Ejecutar: pytest api\tests\unit\equipo\integrante_3_citas\test_integrante_3_citas.py::test_pendiente_puede_pasar_a_agendada
 2. validate_appointment_transition("pending", "scheduled")</t>
         </is>
       </c>
@@ -3294,7 +3291,7 @@
       </c>
       <c r="K18" s="74" t="inlineStr">
         <is>
-          <t>api\tests\unit\equipo\test_integrante_3_citas.py::test_pendiente_puede_pasar_a_agendada -&gt; 1 passed</t>
+          <t>api\tests\unit\equipo\integrante_3_citas\test_integrante_3_citas.py::test_pendiente_puede_pasar_a_agendada -&gt; 1 passed</t>
         </is>
       </c>
       <c r="L18" s="73" t="inlineStr">
@@ -3331,7 +3328,7 @@
       </c>
       <c r="E19" s="73" t="inlineStr">
         <is>
-          <t>1. Ejecutar: pytest api\tests\unit\equipo\test_integrante_3_citas.py::test_agendada_puede_pasar_a_en_progreso
+          <t>1. Ejecutar: pytest api\tests\unit\equipo\integrante_3_citas\test_integrante_3_citas.py::test_agendada_puede_pasar_a_en_progreso
 2. validate_appointment_transition("scheduled", "in_progress")</t>
         </is>
       </c>
@@ -3362,7 +3359,7 @@
       </c>
       <c r="K19" s="74" t="inlineStr">
         <is>
-          <t>api\tests\unit\equipo\test_integrante_3_citas.py::test_agendada_puede_pasar_a_en_progreso -&gt; 1 passed</t>
+          <t>api\tests\unit\equipo\integrante_3_citas\test_integrante_3_citas.py::test_agendada_puede_pasar_a_en_progreso -&gt; 1 passed</t>
         </is>
       </c>
       <c r="L19" s="73" t="inlineStr">
@@ -3399,7 +3396,7 @@
       </c>
       <c r="E20" s="73" t="inlineStr">
         <is>
-          <t>1. Ejecutar: pytest api\tests\unit\equipo\test_integrante_3_citas.py::test_cita_completada_no_puede_cancelarse
+          <t>1. Ejecutar: pytest api\tests\unit\equipo\integrante_3_citas\test_integrante_3_citas.py::test_cita_completada_no_puede_cancelarse
 2. validate_appointment_transition("completed", "cancelled")</t>
         </is>
       </c>
@@ -3430,7 +3427,7 @@
       </c>
       <c r="K20" s="74" t="inlineStr">
         <is>
-          <t>api\tests\unit\equipo\test_integrante_3_citas.py::test_cita_completada_no_puede_cancelarse -&gt; 1 passed</t>
+          <t>api\tests\unit\equipo\integrante_3_citas\test_integrante_3_citas.py::test_cita_completada_no_puede_cancelarse -&gt; 1 passed</t>
         </is>
       </c>
       <c r="L20" s="73" t="inlineStr">
@@ -3467,7 +3464,7 @@
       </c>
       <c r="E21" s="73" t="inlineStr">
         <is>
-          <t>1. Ejecutar: pytest api\tests\unit\equipo\test_integrante_3_citas.py::test_cita_cancelada_no_puede_reabrirse
+          <t>1. Ejecutar: pytest api\tests\unit\equipo\integrante_3_citas\test_integrante_3_citas.py::test_cita_cancelada_no_puede_reabrirse
 2. validate_appointment_transition("cancelled", "scheduled")</t>
         </is>
       </c>
@@ -3498,7 +3495,7 @@
       </c>
       <c r="K21" s="74" t="inlineStr">
         <is>
-          <t>api\tests\unit\equipo\test_integrante_3_citas.py::test_cita_cancelada_no_puede_reabrirse -&gt; 1 passed</t>
+          <t>api\tests\unit\equipo\integrante_3_citas\test_integrante_3_citas.py::test_cita_cancelada_no_puede_reabrirse -&gt; 1 passed</t>
         </is>
       </c>
       <c r="L21" s="73" t="inlineStr">
@@ -3535,7 +3532,7 @@
       </c>
       <c r="E22" s="73" t="inlineStr">
         <is>
-          <t>1. Ejecutar: pytest api\tests\unit\equipo\test_integrante_3_citas.py::test_fecha_invalida_no_genera_horarios
+          <t>1. Ejecutar: pytest api\tests\unit\equipo\integrante_3_citas\test_integrante_3_citas.py::test_fecha_invalida_no_genera_horarios
 2. get_available_time_slots(1, "02-11-2026")</t>
         </is>
       </c>
@@ -3566,7 +3563,7 @@
       </c>
       <c r="K22" s="74" t="inlineStr">
         <is>
-          <t>api\tests\unit\equipo\test_integrante_3_citas.py::test_fecha_invalida_no_genera_horarios -&gt; 1 passed</t>
+          <t>api\tests\unit\equipo\integrante_3_citas\test_integrante_3_citas.py::test_fecha_invalida_no_genera_horarios -&gt; 1 passed</t>
         </is>
       </c>
       <c r="L22" s="73" t="inlineStr">
@@ -3603,7 +3600,7 @@
       </c>
       <c r="E23" s="73" t="inlineStr">
         <is>
-          <t>1. Ejecutar: pytest api\tests\unit\equipo\test_integrante_3_citas.py::test_usuario_que_no_es_tecnico_no_tiene_horarios
+          <t>1. Ejecutar: pytest api\tests\unit\equipo\integrante_3_citas\test_integrante_3_citas.py::test_usuario_que_no_es_tecnico_no_tiene_horarios
 2. get_available_time_slots(cliente.id, "2026-11-02")</t>
         </is>
       </c>
@@ -3634,7 +3631,7 @@
       </c>
       <c r="K23" s="74" t="inlineStr">
         <is>
-          <t>api\tests\unit\equipo\test_integrante_3_citas.py::test_usuario_que_no_es_tecnico_no_tiene_horarios -&gt; 1 passed</t>
+          <t>api\tests\unit\equipo\integrante_3_citas\test_integrante_3_citas.py::test_usuario_que_no_es_tecnico_no_tiene_horarios -&gt; 1 passed</t>
         </is>
       </c>
       <c r="L23" s="73" t="inlineStr">
@@ -3671,7 +3668,7 @@
       </c>
       <c r="E24" s="73" t="inlineStr">
         <is>
-          <t>1. Ejecutar: pytest api\tests\unit\equipo\test_integrante_3_citas.py::test_jornada_laboral_genera_diez_franjas
+          <t>1. Ejecutar: pytest api\tests\unit\equipo\integrante_3_citas\test_integrante_3_citas.py::test_jornada_laboral_genera_diez_franjas
 2. get_available_time_slots(tecnico.id, "2026-11-02")</t>
         </is>
       </c>
@@ -3702,7 +3699,7 @@
       </c>
       <c r="K24" s="74" t="inlineStr">
         <is>
-          <t>api\tests\unit\equipo\test_integrante_3_citas.py::test_jornada_laboral_genera_diez_franjas -&gt; 1 passed</t>
+          <t>api\tests\unit\equipo\integrante_3_citas\test_integrante_3_citas.py::test_jornada_laboral_genera_diez_franjas -&gt; 1 passed</t>
         </is>
       </c>
       <c r="L24" s="73" t="inlineStr">
@@ -3739,7 +3736,7 @@
       </c>
       <c r="E25" s="73" t="inlineStr">
         <is>
-          <t>1. Ejecutar: pytest api\tests\unit\equipo\test_integrante_3_citas.py::test_hora_ocupada_no_se_ofrece
+          <t>1. Ejecutar: pytest api\tests\unit\equipo\integrante_3_citas\test_integrante_3_citas.py::test_hora_ocupada_no_se_ofrece
 2. get_available_time_slots(tecnico.id, "2026-11-02")</t>
         </is>
       </c>
@@ -3770,7 +3767,7 @@
       </c>
       <c r="K25" s="74" t="inlineStr">
         <is>
-          <t>api\tests\unit\equipo\test_integrante_3_citas.py::test_hora_ocupada_no_se_ofrece -&gt; 1 passed</t>
+          <t>api\tests\unit\equipo\integrante_3_citas\test_integrante_3_citas.py::test_hora_ocupada_no_se_ofrece -&gt; 1 passed</t>
         </is>
       </c>
       <c r="L25" s="73" t="inlineStr">
@@ -3807,7 +3804,7 @@
       </c>
       <c r="E26" s="73" t="inlineStr">
         <is>
-          <t>1. Ejecutar: pytest api\tests\unit\equipo\test_integrante_3_citas.py::test_tecnico_libre_esta_disponible
+          <t>1. Ejecutar: pytest api\tests\unit\equipo\integrante_3_citas\test_integrante_3_citas.py::test_tecnico_libre_esta_disponible
 2. check_technician_availability(tecnico.id, "2026-11-02", "09:00")</t>
         </is>
       </c>
@@ -3838,7 +3835,7 @@
       </c>
       <c r="K26" s="74" t="inlineStr">
         <is>
-          <t>api\tests\unit\equipo\test_integrante_3_citas.py::test_tecnico_libre_esta_disponible -&gt; 1 passed</t>
+          <t>api\tests\unit\equipo\integrante_3_citas\test_integrante_3_citas.py::test_tecnico_libre_esta_disponible -&gt; 1 passed</t>
         </is>
       </c>
       <c r="L26" s="73" t="inlineStr">
@@ -3875,7 +3872,7 @@
       </c>
       <c r="E27" s="73" t="inlineStr">
         <is>
-          <t>1. Ejecutar: pytest api\tests\unit\equipo\test_integrante_3_citas.py::test_tecnico_fuera_de_horario_no_esta_disponible
+          <t>1. Ejecutar: pytest api\tests\unit\equipo\integrante_3_citas\test_integrante_3_citas.py::test_tecnico_fuera_de_horario_no_esta_disponible
 2. check_technician_availability(tecnico.id, "2026-11-02", "07:00")</t>
         </is>
       </c>
@@ -3906,7 +3903,7 @@
       </c>
       <c r="K27" s="74" t="inlineStr">
         <is>
-          <t>api\tests\unit\equipo\test_integrante_3_citas.py::test_tecnico_fuera_de_horario_no_esta_disponible -&gt; 1 passed</t>
+          <t>api\tests\unit\equipo\integrante_3_citas\test_integrante_3_citas.py::test_tecnico_fuera_de_horario_no_esta_disponible -&gt; 1 passed</t>
         </is>
       </c>
       <c r="L27" s="73" t="inlineStr">

</xml_diff>